<commit_message>
[1.1.0.24] Improved & stable Version of FKZ-Performer
</commit_message>
<xml_diff>
--- a/Prod/rpa003_FKZ_Performer/Data/Config.xlsx
+++ b/Prod/rpa003_FKZ_Performer/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baris.isik\develop\rpa\uipath-rpa_fkz\Prod\rpa003_FKZ_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9156C7A2-D900-4A14-927E-A698383D66D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51B12B4-38D7-4928-A476-6939A6B34E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="52">
   <si>
     <t>Name</t>
   </si>
@@ -34,39 +34,6 @@
   </si>
   <si>
     <t>MaxRetryNumber</t>
-  </si>
-  <si>
-    <t>LogMessage_GetTransactionData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Processing Transaction Number: </t>
-  </si>
-  <si>
-    <t>LogMessage_GetTransactionDataError</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
-  </si>
-  <si>
-    <t>Static part of logging message. Error retrieving Transaction Data.</t>
-  </si>
-  <si>
-    <t>LogMessage_Success</t>
-  </si>
-  <si>
-    <t>Transaction Successful.</t>
-  </si>
-  <si>
-    <t>LogMessage_BusinessRuleException</t>
-  </si>
-  <si>
-    <t>Business rule exception.</t>
-  </si>
-  <si>
-    <t>LogMessage_ApplicationException</t>
-  </si>
-  <si>
-    <t>System exception.</t>
   </si>
   <si>
     <t>logF_BusinessProcessName</t>
@@ -83,18 +50,6 @@
     <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
   </si>
   <si>
-    <t>Static part of logging message. Processed Transaction succesful.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Processed Transaction failed with business exception.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Processed Transaction failed with application exception.</t>
-  </si>
-  <si>
-    <t>Static part of logging message. Calling Get Transaction Data.</t>
-  </si>
-  <si>
     <t>OrchestratorQueueFolder</t>
   </si>
   <si>
@@ -104,18 +59,12 @@
     <t>MaxConsecutiveSystemExceptions</t>
   </si>
   <si>
-    <t>ExceptionMessage_ConsecutiveErrors</t>
-  </si>
-  <si>
     <t>RetryNumberGetTransactionItem</t>
   </si>
   <si>
     <t>RetryNumberSetTransactionStatus</t>
   </si>
   <si>
-    <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
-  </si>
-  <si>
     <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
   </si>
   <si>
@@ -131,9 +80,6 @@
     <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
   </si>
   <si>
-    <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
-  </si>
-  <si>
     <t>OrchestratorQueueName</t>
   </si>
   <si>
@@ -221,9 +167,6 @@
     <t>rpa003_Queue_Main</t>
   </si>
   <si>
-    <t>rpa003_Duration_AvgPerItem</t>
-  </si>
-  <si>
     <t>rpa003_Mailbox_Business</t>
   </si>
   <si>
@@ -231,6 +174,12 @@
   </si>
   <si>
     <t>rpa003_SAP_ConnectionName</t>
+  </si>
+  <si>
+    <t>ObsMaxAttemptsPerSession</t>
+  </si>
+  <si>
+    <t>rpa003_Duration_AvgProcessing</t>
   </si>
 </sst>
 </file>
@@ -289,18 +238,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -618,20 +578,20 @@
   <dimension ref="A1:Z996"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="43" style="5" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" style="5" customWidth="1"/>
     <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1"/>
@@ -659,50 +619,52 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
+      <c r="A2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="43.2">
-      <c r="A3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="4" t="s">
-        <v>24</v>
+      <c r="A3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="28.8">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>17</v>
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" t="s">
-        <v>43</v>
+      <c r="A7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" t="s">
-        <v>58</v>
+      <c r="A8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1702,23 +1664,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z966"/>
+  <dimension ref="A1:Z958"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="64.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="1" max="1" width="41" style="5" customWidth="1"/>
+    <col min="2" max="2" width="64.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" style="5" customWidth="1"/>
     <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1"/>
@@ -1746,223 +1708,170 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="28.8">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="5">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>18</v>
+      <c r="C2" s="7" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="43.2">
-      <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3">
+      <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5">
         <v>0</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>33</v>
+      <c r="C3" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5">
+        <v>2</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>22</v>
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
+    <row r="7" spans="1:26" ht="28.8">
+      <c r="A7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
+    <row r="8" spans="1:26" ht="14.4">
+      <c r="C8" s="7"/>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
+      <c r="A9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="5">
+        <v>587</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="A10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="5">
+        <v>300</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>30</v>
+      <c r="A12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="s">
-        <v>31</v>
-      </c>
+      <c r="B13" s="6"/>
     </row>
-    <row r="14" spans="1:26" ht="28.8">
-      <c r="A14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>34</v>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.4">
-      <c r="C15" s="3"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16">
-        <v>587</v>
+      <c r="A16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B17" t="s">
-        <v>39</v>
-      </c>
     </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A18" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18">
+    <row r="18" spans="1:3" ht="15" customHeight="1">
+      <c r="A18" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15" customHeight="1">
+      <c r="A20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="5">
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A24" t="s">
-        <v>49</v>
-      </c>
-      <c r="B24" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="15" customHeight="1">
-      <c r="A25" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" t="s">
-        <v>56</v>
-      </c>
-    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2893,14 +2802,6 @@
     <row r="956" ht="14.25" customHeight="1"/>
     <row r="957" ht="14.25" customHeight="1"/>
     <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2909,7 +2810,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D972"/>
+  <dimension ref="A1:D969"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
@@ -2918,100 +2819,86 @@
     <col min="4" max="26" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1" ht="15" customHeight="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:4" s="3" customFormat="1" ht="15" customHeight="1">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" t="s">
-        <v>68</v>
-      </c>
-    </row>
+    <row r="10" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:4" ht="14.25" customHeight="1"/>
@@ -3970,9 +3857,6 @@
     <row r="967" ht="14.25" customHeight="1"/>
     <row r="968" ht="14.25" customHeight="1"/>
     <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>